<commit_message>
Final fixes before submission
</commit_message>
<xml_diff>
--- a/outputs/laicpms_final.xlsx
+++ b/outputs/laicpms_final.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV48"/>
+  <dimension ref="A1:AU48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -652,11 +652,6 @@
       </c>
       <c r="AU1" t="inlineStr">
         <is>
-          <t>Pb/Pb*</t>
-        </is>
-      </c>
-      <c r="AV1" t="inlineStr">
-        <is>
           <t>Pb_contaminated</t>
         </is>
       </c>
@@ -806,10 +801,7 @@
       <c r="AT2" t="n">
         <v>2.053360512993144</v>
       </c>
-      <c r="AU2" t="n">
-        <v>1.04365751532534</v>
-      </c>
-      <c r="AV2" t="b">
+      <c r="AU2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -958,10 +950,7 @@
       <c r="AT3" t="n">
         <v>1.384740007937938</v>
       </c>
-      <c r="AU3" t="n">
-        <v>0.729985524379383</v>
-      </c>
-      <c r="AV3" t="b">
+      <c r="AU3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1110,10 +1099,7 @@
       <c r="AT4" t="n">
         <v>1.273528919609876</v>
       </c>
-      <c r="AU4" t="n">
-        <v>1.179010154761562</v>
-      </c>
-      <c r="AV4" t="b">
+      <c r="AU4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1262,10 +1248,7 @@
       <c r="AT5" t="n">
         <v>2.260195362223512</v>
       </c>
-      <c r="AU5" t="n">
-        <v>0.3863571060573424</v>
-      </c>
-      <c r="AV5" t="b">
+      <c r="AU5" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1414,10 +1397,7 @@
       <c r="AT6" t="n">
         <v>2.071939005139642</v>
       </c>
-      <c r="AU6" t="n">
-        <v>1.352865902892808</v>
-      </c>
-      <c r="AV6" t="b">
+      <c r="AU6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1566,10 +1546,7 @@
       <c r="AT7" t="n">
         <v>1.797686251925831</v>
       </c>
-      <c r="AU7" t="n">
-        <v>1.589459032915284</v>
-      </c>
-      <c r="AV7" t="b">
+      <c r="AU7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1718,10 +1695,7 @@
       <c r="AT8" t="n">
         <v>1.059486301810651</v>
       </c>
-      <c r="AU8" t="n">
-        <v>12.4118196513188</v>
-      </c>
-      <c r="AV8" t="b">
+      <c r="AU8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1870,10 +1844,7 @@
       <c r="AT9" t="n">
         <v>1.618919438569506</v>
       </c>
-      <c r="AU9" t="n">
-        <v>0.3516397691704972</v>
-      </c>
-      <c r="AV9" t="b">
+      <c r="AU9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2022,10 +1993,7 @@
       <c r="AT10" t="n">
         <v>1.48689060098437</v>
       </c>
-      <c r="AU10" t="n">
-        <v>17.87863546289187</v>
-      </c>
-      <c r="AV10" t="b">
+      <c r="AU10" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2174,10 +2142,7 @@
       <c r="AT11" t="n">
         <v>1.997973794745482</v>
       </c>
-      <c r="AU11" t="n">
-        <v>0.3102438692617022</v>
-      </c>
-      <c r="AV11" t="b">
+      <c r="AU11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2326,10 +2291,7 @@
       <c r="AT12" t="n">
         <v>1.802636690612446</v>
       </c>
-      <c r="AU12" t="n">
-        <v>0.4210033283566933</v>
-      </c>
-      <c r="AV12" t="b">
+      <c r="AU12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2478,10 +2440,7 @@
       <c r="AT13" t="n">
         <v>1.022273891578807</v>
       </c>
-      <c r="AU13" t="n">
-        <v>8.663196229620421</v>
-      </c>
-      <c r="AV13" t="b">
+      <c r="AU13" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2630,10 +2589,7 @@
       <c r="AT14" t="n">
         <v>1.350129732632996</v>
       </c>
-      <c r="AU14" t="n">
-        <v>0.2864888729659009</v>
-      </c>
-      <c r="AV14" t="b">
+      <c r="AU14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2782,10 +2738,7 @@
       <c r="AT15" t="n">
         <v>0.9233534647536576</v>
       </c>
-      <c r="AU15" t="n">
-        <v>27.15124324012993</v>
-      </c>
-      <c r="AV15" t="b">
+      <c r="AU15" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2934,10 +2887,7 @@
       <c r="AT16" t="n">
         <v>2.331039126517843</v>
       </c>
-      <c r="AU16" t="n">
-        <v>0.4311337307247004</v>
-      </c>
-      <c r="AV16" t="b">
+      <c r="AU16" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3086,10 +3036,7 @@
       <c r="AT17" t="n">
         <v>1.660756207760848</v>
       </c>
-      <c r="AU17" t="n">
-        <v>0.608530097241759</v>
-      </c>
-      <c r="AV17" t="b">
+      <c r="AU17" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3238,10 +3185,7 @@
       <c r="AT18" t="n">
         <v>2.333882831423486</v>
       </c>
-      <c r="AU18" t="n">
-        <v>0.3364034412201939</v>
-      </c>
-      <c r="AV18" t="b">
+      <c r="AU18" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3390,10 +3334,7 @@
       <c r="AT19" t="n">
         <v>1.423319100356607</v>
       </c>
-      <c r="AU19" t="n">
-        <v>6.884575329139084</v>
-      </c>
-      <c r="AV19" t="b">
+      <c r="AU19" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3542,10 +3483,7 @@
       <c r="AT20" t="n">
         <v>1.189405306562669</v>
       </c>
-      <c r="AU20" t="n">
-        <v>6.091322080301743</v>
-      </c>
-      <c r="AV20" t="b">
+      <c r="AU20" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3694,10 +3632,7 @@
       <c r="AT21" t="n">
         <v>0.3793523088060705</v>
       </c>
-      <c r="AU21" t="n">
-        <v>0.9920531218713348</v>
-      </c>
-      <c r="AV21" t="b">
+      <c r="AU21" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3846,10 +3781,7 @@
       <c r="AT22" t="n">
         <v>1.384824506638552</v>
       </c>
-      <c r="AU22" t="n">
-        <v>2.008008681394003</v>
-      </c>
-      <c r="AV22" t="b">
+      <c r="AU22" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3998,10 +3930,7 @@
       <c r="AT23" t="n">
         <v>3.007796361494169</v>
       </c>
-      <c r="AU23" t="n">
-        <v>0.4969227527060488</v>
-      </c>
-      <c r="AV23" t="b">
+      <c r="AU23" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4150,10 +4079,7 @@
       <c r="AT24" t="n">
         <v>0.8905195332522047</v>
       </c>
-      <c r="AU24" t="n">
-        <v>0.4387152276367237</v>
-      </c>
-      <c r="AV24" t="b">
+      <c r="AU24" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4302,10 +4228,7 @@
       <c r="AT25" t="n">
         <v>5.820350045681135</v>
       </c>
-      <c r="AU25" t="n">
-        <v>0.7129752948273733</v>
-      </c>
-      <c r="AV25" t="b">
+      <c r="AU25" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4454,10 +4377,7 @@
       <c r="AT26" t="n">
         <v>2.714521648814483</v>
       </c>
-      <c r="AU26" t="n">
-        <v>0.2787730964307529</v>
-      </c>
-      <c r="AV26" t="b">
+      <c r="AU26" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4606,10 +4526,7 @@
       <c r="AT27" t="n">
         <v>2.473129117774863</v>
       </c>
-      <c r="AU27" t="n">
-        <v>0.3187657538160178</v>
-      </c>
-      <c r="AV27" t="b">
+      <c r="AU27" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4758,10 +4675,7 @@
       <c r="AT28" t="n">
         <v>3.271611980014718</v>
       </c>
-      <c r="AU28" t="n">
-        <v>0.4230002216926091</v>
-      </c>
-      <c r="AV28" t="b">
+      <c r="AU28" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4910,10 +4824,7 @@
       <c r="AT29" t="n">
         <v>1.253126028174256</v>
       </c>
-      <c r="AU29" t="n">
-        <v>0.6698231052795961</v>
-      </c>
-      <c r="AV29" t="b">
+      <c r="AU29" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5062,10 +4973,7 @@
       <c r="AT30" t="n">
         <v>1.497232175443367</v>
       </c>
-      <c r="AU30" t="n">
-        <v>0.5096504627644629</v>
-      </c>
-      <c r="AV30" t="b">
+      <c r="AU30" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5214,10 +5122,7 @@
       <c r="AT31" t="n">
         <v>2.621070839991518</v>
       </c>
-      <c r="AU31" t="n">
-        <v>1.175427175585403</v>
-      </c>
-      <c r="AV31" t="b">
+      <c r="AU31" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5366,10 +5271,7 @@
       <c r="AT32" t="n">
         <v>1.420879374261057</v>
       </c>
-      <c r="AU32" t="n">
-        <v>0.3373214963452137</v>
-      </c>
-      <c r="AV32" t="b">
+      <c r="AU32" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5518,10 +5420,7 @@
       <c r="AT33" t="n">
         <v>1.265519454952096</v>
       </c>
-      <c r="AU33" t="n">
-        <v>0.3847925815930527</v>
-      </c>
-      <c r="AV33" t="b">
+      <c r="AU33" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5670,10 +5569,7 @@
       <c r="AT34" t="n">
         <v>2.099037529517763</v>
       </c>
-      <c r="AU34" t="n">
-        <v>0.3598467851879865</v>
-      </c>
-      <c r="AV34" t="b">
+      <c r="AU34" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5822,10 +5718,7 @@
       <c r="AT35" t="n">
         <v>1.414082454040926</v>
       </c>
-      <c r="AU35" t="n">
-        <v>0.3985054394240253</v>
-      </c>
-      <c r="AV35" t="b">
+      <c r="AU35" t="b">
         <v>0</v>
       </c>
     </row>
@@ -5974,10 +5867,7 @@
       <c r="AT36" t="n">
         <v>2.529107763586727</v>
       </c>
-      <c r="AU36" t="n">
-        <v>0.45708704441798</v>
-      </c>
-      <c r="AV36" t="b">
+      <c r="AU36" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6126,10 +6016,7 @@
       <c r="AT37" t="n">
         <v>1.369023525433005</v>
       </c>
-      <c r="AU37" t="n">
-        <v>0.717361802015832</v>
-      </c>
-      <c r="AV37" t="b">
+      <c r="AU37" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6278,10 +6165,7 @@
       <c r="AT38" t="n">
         <v>1.538972937162101</v>
       </c>
-      <c r="AU38" t="n">
-        <v>0.455824610737244</v>
-      </c>
-      <c r="AV38" t="b">
+      <c r="AU38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6430,10 +6314,7 @@
       <c r="AT39" t="n">
         <v>1.539675569283793</v>
       </c>
-      <c r="AU39" t="n">
-        <v>0.451524442119231</v>
-      </c>
-      <c r="AV39" t="b">
+      <c r="AU39" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6582,10 +6463,7 @@
       <c r="AT40" t="n">
         <v>1.407497340538534</v>
       </c>
-      <c r="AU40" t="n">
-        <v>0.3758838331591971</v>
-      </c>
-      <c r="AV40" t="b">
+      <c r="AU40" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6734,10 +6612,7 @@
       <c r="AT41" t="n">
         <v>1.485031870595837</v>
       </c>
-      <c r="AU41" t="n">
-        <v>0.4128549634238162</v>
-      </c>
-      <c r="AV41" t="b">
+      <c r="AU41" t="b">
         <v>0</v>
       </c>
     </row>
@@ -6886,10 +6761,7 @@
       <c r="AT42" t="n">
         <v>1.303595632819731</v>
       </c>
-      <c r="AU42" t="n">
-        <v>6.390201692323537</v>
-      </c>
-      <c r="AV42" t="b">
+      <c r="AU42" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7038,10 +6910,7 @@
       <c r="AT43" t="n">
         <v>2.096414758394205</v>
       </c>
-      <c r="AU43" t="n">
-        <v>73.24654835279628</v>
-      </c>
-      <c r="AV43" t="b">
+      <c r="AU43" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7190,10 +7059,7 @@
       <c r="AT44" t="n">
         <v>0.912655311295953</v>
       </c>
-      <c r="AU44" t="n">
-        <v>0.4361821518895005</v>
-      </c>
-      <c r="AV44" t="b">
+      <c r="AU44" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7342,10 +7208,7 @@
       <c r="AT45" t="n">
         <v>1.436191048508687</v>
       </c>
-      <c r="AU45" t="n">
-        <v>0.4130868347963643</v>
-      </c>
-      <c r="AV45" t="b">
+      <c r="AU45" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7494,10 +7357,7 @@
       <c r="AT46" t="n">
         <v>2.502021493960294</v>
       </c>
-      <c r="AU46" t="n">
-        <v>104.0838075337448</v>
-      </c>
-      <c r="AV46" t="b">
+      <c r="AU46" t="b">
         <v>1</v>
       </c>
     </row>
@@ -7646,10 +7506,7 @@
       <c r="AT47" t="n">
         <v>2.873365343297738</v>
       </c>
-      <c r="AU47" t="n">
-        <v>0.3972726183017091</v>
-      </c>
-      <c r="AV47" t="b">
+      <c r="AU47" t="b">
         <v>0</v>
       </c>
     </row>
@@ -7798,10 +7655,7 @@
       <c r="AT48" t="n">
         <v>1.528121703414548</v>
       </c>
-      <c r="AU48" t="n">
-        <v>0.7239141452766381</v>
-      </c>
-      <c r="AV48" t="b">
+      <c r="AU48" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>